<commit_message>
Russian and Chinese translations, Millbrook, click finishes typing
- Imported all translated pieces into translations/ru.po and zh_CN.po.
- Translate before uppercasing / unquoting / first-name splitting; add
  MOVES and TIP.
- Rename the town Duskhaven -> Millbrook (English and both translations).
- Dialogue: a click during typing kills the typing tween, so the line
  stays whole.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TeVA9WJDfvrL1N6Qe3Kpqx
</commit_message>
<xml_diff>
--- a/docs/voice/Charm_Combo_Voice_Script.xlsx
+++ b/docs/voice/Charm_Combo_Voice_Script.xlsx
@@ -845,7 +845,7 @@
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>Amara = ah-MAH-ruh · Duskrose = DUSK-rose · Duskhaven = DUSK-hay-vun · grimoire = grim-WAHR</t>
+          <t>Amara = ah-MAH-ruh · Duskrose = DUSK-rose · Millbrook = MILL-brook · grimoire = grim-WAHR</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Opal, slime. An adult who spent thirty-one years hiding in a jar in the woods north of Duskhaven, listening to people on the path. Soft, polite, a little formal; stutters on the first word when she's nervous, apologises and then corrects herself. Very exact about her collection (counts, where each thing came from). Gets braver and funnier as the story goes on. Shy, never childish.</t>
+          <t>Opal, slime. An adult who spent thirty-one years hiding in a jar in the woods north of Millbrook, listening to people on the path. Soft, polite, a little formal; stutters on the first word when she's nervous, apologises and then corrects herself. Very exact about her collection (counts, where each thing came from). Gets braver and funnier as the story goes on. Shy, never childish.</t>
         </is>
       </c>
     </row>
@@ -972,7 +972,7 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Say it: Amara = ah-MAH-ruh · Duskrose = DUSK-rose · Duskhaven = DUSK-hay-vun · grimoire = grim-WAHR</t>
+          <t>Say it: Amara = ah-MAH-ruh · Duskrose = DUSK-rose · Millbrook = MILL-brook · grimoire = grim-WAHR</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
     <row r="2" ht="44" customHeight="1">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Opal, slime. An adult who spent thirty-one years hiding in a jar in the woods north of Duskhaven, listening to people on the path. Soft, polite, a little formal; stutters on the first word when she's nervous, apologises and then corrects herself. Very exact about her collection (counts, where each thing came from). Gets braver and funnier as the story goes on. Shy, never childish.</t>
+          <t>Opal, slime. An adult who spent thirty-one years hiding in a jar in the woods north of Millbrook, listening to people on the path. Soft, polite, a little formal; stutters on the first word when she's nervous, apologises and then corrects herself. Very exact about her collection (counts, where each thing came from). Gets braver and funnier as the story goes on. Shy, never childish.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Match Hazel's and Marina's expressions to their lines
Hazel's "teasing" picture is a lip-bite, so it now marks flirting only;
dry jokes go neutral, jealousy angry, mischief happy, tender lines shy
(12 lines). Marina: 5 lines. Editing guide gets an expression table.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TeVA9WJDfvrL1N6Qe3Kpqx
</commit_message>
<xml_diff>
--- a/docs/voice/Charm_Combo_Voice_Script.xlsx
+++ b/docs/voice/Charm_Combo_Voice_Script.xlsx
@@ -4400,7 +4400,7 @@
       </c>
       <c r="G8" s="24" t="inlineStr">
         <is>
-          <t>angry</t>
+          <t>shy</t>
         </is>
       </c>
       <c r="H8" s="24" t="inlineStr">
@@ -4862,7 +4862,7 @@
       </c>
       <c r="G19" s="27" t="inlineStr">
         <is>
-          <t>teasing</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="H19" s="27" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="G39" s="27" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>shy</t>
         </is>
       </c>
       <c r="H39" s="27" t="inlineStr">
@@ -11084,7 +11084,7 @@
       </c>
       <c r="G10" s="24" t="inlineStr">
         <is>
-          <t>teasing</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="H10" s="24" t="inlineStr">
@@ -11294,7 +11294,7 @@
       </c>
       <c r="G15" s="27" t="inlineStr">
         <is>
-          <t>teasing</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="H15" s="27" t="inlineStr">
@@ -11378,7 +11378,7 @@
       </c>
       <c r="G17" s="27" t="inlineStr">
         <is>
-          <t>teasing</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="H17" s="27" t="inlineStr">
@@ -11588,7 +11588,7 @@
       </c>
       <c r="G22" s="24" t="inlineStr">
         <is>
-          <t>teasing</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="H22" s="24" t="inlineStr">
@@ -11672,7 +11672,7 @@
       </c>
       <c r="G24" s="24" t="inlineStr">
         <is>
-          <t>teasing</t>
+          <t>angry</t>
         </is>
       </c>
       <c r="H24" s="24" t="inlineStr">
@@ -11756,7 +11756,7 @@
       </c>
       <c r="G26" s="24" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>shy</t>
         </is>
       </c>
       <c r="H26" s="24" t="inlineStr">
@@ -12176,7 +12176,7 @@
       </c>
       <c r="G36" s="24" t="inlineStr">
         <is>
-          <t>teasing</t>
+          <t>happy</t>
         </is>
       </c>
       <c r="H36" s="24" t="inlineStr">
@@ -12470,7 +12470,7 @@
       </c>
       <c r="G43" s="27" t="inlineStr">
         <is>
-          <t>teasing</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="H43" s="27" t="inlineStr">
@@ -12554,7 +12554,7 @@
       </c>
       <c r="G45" s="27" t="inlineStr">
         <is>
-          <t>teasing</t>
+          <t>shy</t>
         </is>
       </c>
       <c r="H45" s="27" t="inlineStr">
@@ -12680,7 +12680,7 @@
       </c>
       <c r="G48" s="24" t="inlineStr">
         <is>
-          <t>teasing</t>
+          <t>happy</t>
         </is>
       </c>
       <c r="H48" s="24" t="inlineStr">
@@ -12890,7 +12890,7 @@
       </c>
       <c r="G53" s="27" t="inlineStr">
         <is>
-          <t>teasing</t>
+          <t>happy</t>
         </is>
       </c>
       <c r="H53" s="27" t="inlineStr">

</xml_diff>

<commit_message>
Marina's recorded script and 78 voice clips; gameplay badges from the packs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TeVA9WJDfvrL1N6Qe3Kpqx
</commit_message>
<xml_diff>
--- a/docs/voice/Charm_Combo_Voice_Script.xlsx
+++ b/docs/voice/Charm_Combo_Voice_Script.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Amara'!$A$5:$J$79</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Amara'!$5:$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Marina'!$A$5:$J$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Marina'!$A$5:$J$79</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Marina'!$5:$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Opal'!$A$5:$J$79</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Opal'!$5:$5</definedName>
@@ -4177,7 +4177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J82"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4353,7 +4353,7 @@
       </c>
       <c r="F7" s="28" t="inlineStr">
         <is>
-          <t>Nerissa. Don't. Don't you dare.</t>
+          <t>Don't. Don't you dare.</t>
         </is>
       </c>
       <c r="G7" s="27" t="inlineStr">
@@ -4390,12 +4390,12 @@
       </c>
       <c r="E8" s="23" t="inlineStr">
         <is>
-          <t>Her previous line: Nerissa. Don't. Don't you dare.</t>
+          <t>Her previous line: Don't. Don't you dare.</t>
         </is>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>Gran, I'm fine. I was resting. I always rest like that.</t>
+          <t>Gran, I'm fine. I'm always like that.</t>
         </is>
       </c>
       <c r="G8" s="24" t="inlineStr">
@@ -4605,7 +4605,7 @@
       </c>
       <c r="F13" s="28" t="inlineStr">
         <is>
-          <t>And you're not going to tell anyone either, are you, lifeguard.</t>
+          <t>And you're not going to tell anyone either, are you, lifeguard?</t>
         </is>
       </c>
       <c r="G13" s="27" t="inlineStr">
@@ -4773,7 +4773,7 @@
       </c>
       <c r="F17" s="28" t="inlineStr">
         <is>
-          <t>There. Now we're even. Low tide's at six. Bring your other shoe.</t>
+          <t>There. Now we're even. Low tide's at six.</t>
         </is>
       </c>
       <c r="G17" s="27" t="inlineStr">
@@ -5193,7 +5193,7 @@
       </c>
       <c r="F27" s="28" t="inlineStr">
         <is>
-          <t>Nerissa keeps asking about the comb. I keep saying it's at the jeweller's. I'm running out of jewellers.</t>
+          <t>Everyone keeps asking about the comb and I'm running out of excuses.</t>
         </is>
       </c>
       <c r="G27" s="27" t="inlineStr">
@@ -5487,7 +5487,7 @@
       </c>
       <c r="F34" s="25" t="inlineStr">
         <is>
-          <t>You're a genius, you're a soaked genius with one shoe, come here.</t>
+          <t>You're a genius, you're a soaked genius.</t>
         </is>
       </c>
       <c r="G34" s="24" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="F54" s="25" t="inlineStr">
         <is>
-          <t>So. Last night. I've been floating here trying to think of a word for it, and I've got it down to three, and they're all very rude.</t>
+          <t>So. Last night. I've been floating close by trying to think of a word for it, and I've got it down to three, and they're all very rude.</t>
         </is>
       </c>
       <c r="G54" s="24" t="inlineStr">
@@ -6343,7 +6343,7 @@
       <c r="I54" s="24" t="n"/>
       <c r="J54" s="24" t="n"/>
     </row>
-    <row r="55" ht="54" customHeight="1">
+    <row r="55" ht="67.5" customHeight="1">
       <c r="A55" s="26" t="n">
         <v>50</v>
       </c>
@@ -6364,7 +6364,7 @@
       </c>
       <c r="E55" s="26" t="inlineStr">
         <is>
-          <t>Her previous line: So. Last night. I've been floating here trying to think of a word for it, and I've got it down to three, and they're all very rude.</t>
+          <t>Her previous line: So. Last night. I've been floating close by trying to think of a word for it, and I've got it down to three, and they're all very rude.</t>
         </is>
       </c>
       <c r="F55" s="28" t="inlineStr">
@@ -6453,7 +6453,7 @@
       </c>
       <c r="F57" s="28" t="inlineStr">
         <is>
-          <t>Dance with me later. Badly. I've got a tail, so we'll be bad at it together.</t>
+          <t>Swim with me later. Don't embarrass me again.</t>
         </is>
       </c>
       <c r="G57" s="27" t="inlineStr">
@@ -6469,7 +6469,7 @@
       <c r="I57" s="27" t="n"/>
       <c r="J57" s="27" t="n"/>
     </row>
-    <row r="58" ht="40.5" customHeight="1">
+    <row r="58" ht="27" customHeight="1">
       <c r="A58" s="23" t="n">
         <v>53</v>
       </c>
@@ -6490,7 +6490,7 @@
       </c>
       <c r="E58" s="23" t="inlineStr">
         <is>
-          <t>Her previous line: Dance with me later. Badly. I've got a tail, so we'll be bad at it together.</t>
+          <t>Her previous line: Swim with me later. Don't embarrass me again.</t>
         </is>
       </c>
       <c r="F58" s="25" t="inlineStr">
@@ -6979,12 +6979,12 @@
       </c>
       <c r="B70" s="24" t="inlineStr">
         <is>
-          <t>marina_least_01</t>
+          <t>marina_least_02</t>
         </is>
       </c>
       <c r="C70" s="23" t="inlineStr">
         <is>
-          <t>marina_least_01.wav</t>
+          <t>marina_least_02.wav</t>
         </is>
       </c>
       <c r="D70" s="25" t="inlineStr">
@@ -6999,7 +6999,7 @@
       </c>
       <c r="F70" s="25" t="inlineStr">
         <is>
-          <t>Who brings fire to a pier?</t>
+          <t>Ugh. That's drier than a sponge.</t>
         </is>
       </c>
       <c r="G70" s="24" t="inlineStr">
@@ -7009,7 +7009,7 @@
       </c>
       <c r="H70" s="24" t="inlineStr">
         <is>
-          <t>Sarcastic, baffled.</t>
+          <t>Disgusted, then guilty about Gran.</t>
         </is>
       </c>
       <c r="I70" s="24" t="n"/>
@@ -7021,12 +7021,12 @@
       </c>
       <c r="B71" s="27" t="inlineStr">
         <is>
-          <t>marina_least_02</t>
+          <t>marina_least_03</t>
         </is>
       </c>
       <c r="C71" s="26" t="inlineStr">
         <is>
-          <t>marina_least_02.wav</t>
+          <t>marina_least_03.wav</t>
         </is>
       </c>
       <c r="D71" s="27" t="inlineStr">
@@ -7041,7 +7041,7 @@
       </c>
       <c r="F71" s="28" t="inlineStr">
         <is>
-          <t>Ugh. That's drier than Gran's sponge.</t>
+          <t>No. Absolutely not.</t>
         </is>
       </c>
       <c r="G71" s="27" t="inlineStr">
@@ -7051,7 +7051,7 @@
       </c>
       <c r="H71" s="27" t="inlineStr">
         <is>
-          <t>Disgusted, then guilty about Gran.</t>
+          <t>Flat refusal.</t>
         </is>
       </c>
       <c r="I71" s="27" t="n"/>
@@ -7063,12 +7063,12 @@
       </c>
       <c r="B72" s="24" t="inlineStr">
         <is>
-          <t>marina_least_03</t>
+          <t>marina_least_04</t>
         </is>
       </c>
       <c r="C72" s="23" t="inlineStr">
         <is>
-          <t>marina_least_03.wav</t>
+          <t>marina_least_04.wav</t>
         </is>
       </c>
       <c r="D72" s="24" t="inlineStr">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="F72" s="25" t="inlineStr">
         <is>
-          <t>No. Absolutely not.</t>
+          <t>Who even likes those?</t>
         </is>
       </c>
       <c r="G72" s="24" t="inlineStr">
@@ -7093,7 +7093,7 @@
       </c>
       <c r="H72" s="24" t="inlineStr">
         <is>
-          <t>Flat refusal.</t>
+          <t>Genuinely baffled.</t>
         </is>
       </c>
       <c r="I72" s="24" t="n"/>
@@ -7105,12 +7105,12 @@
       </c>
       <c r="B73" s="27" t="inlineStr">
         <is>
-          <t>marina_least_04</t>
+          <t>marina_least_05</t>
         </is>
       </c>
       <c r="C73" s="26" t="inlineStr">
         <is>
-          <t>marina_least_04.wav</t>
+          <t>marina_least_05.wav</t>
         </is>
       </c>
       <c r="D73" s="27" t="inlineStr">
@@ -7125,7 +7125,7 @@
       </c>
       <c r="F73" s="28" t="inlineStr">
         <is>
-          <t>Who even likes those?</t>
+          <t>That's a dry-land gem. Put it back.</t>
         </is>
       </c>
       <c r="G73" s="27" t="inlineStr">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="H73" s="27" t="inlineStr">
         <is>
-          <t>Genuinely baffled.</t>
+          <t>Bossy.</t>
         </is>
       </c>
       <c r="I73" s="27" t="n"/>
@@ -7147,17 +7147,17 @@
       </c>
       <c r="B74" s="24" t="inlineStr">
         <is>
-          <t>marina_least_05</t>
+          <t>marina_chat_01</t>
         </is>
       </c>
       <c r="C74" s="23" t="inlineStr">
         <is>
-          <t>marina_least_05.wav</t>
-        </is>
-      </c>
-      <c r="D74" s="24" t="inlineStr">
-        <is>
-          <t>Puzzle quip: you matched a gem she dislikes</t>
+          <t>marina_chat_01.wav</t>
+        </is>
+      </c>
+      <c r="D74" s="25" t="inlineStr">
+        <is>
+          <t>Puzzle quip: chatter while you play</t>
         </is>
       </c>
       <c r="E74" s="23" t="inlineStr">
@@ -7167,7 +7167,7 @@
       </c>
       <c r="F74" s="25" t="inlineStr">
         <is>
-          <t>That's a dry-land gem. Put it back.</t>
+          <t>Nine days. Keep going.</t>
         </is>
       </c>
       <c r="G74" s="24" t="inlineStr">
@@ -7177,7 +7177,7 @@
       </c>
       <c r="H74" s="24" t="inlineStr">
         <is>
-          <t>Bossy.</t>
+          <t>Tense, focused.</t>
         </is>
       </c>
       <c r="I74" s="24" t="n"/>
@@ -7189,15 +7189,15 @@
       </c>
       <c r="B75" s="27" t="inlineStr">
         <is>
-          <t>marina_chat_01</t>
+          <t>marina_chat_02</t>
         </is>
       </c>
       <c r="C75" s="26" t="inlineStr">
         <is>
-          <t>marina_chat_01.wav</t>
-        </is>
-      </c>
-      <c r="D75" s="28" t="inlineStr">
+          <t>marina_chat_02.wav</t>
+        </is>
+      </c>
+      <c r="D75" s="27" t="inlineStr">
         <is>
           <t>Puzzle quip: chatter while you play</t>
         </is>
@@ -7209,7 +7209,7 @@
       </c>
       <c r="F75" s="28" t="inlineStr">
         <is>
-          <t>Nine days. Keep going.</t>
+          <t>You're getting good at this. It's annoying.</t>
         </is>
       </c>
       <c r="G75" s="27" t="inlineStr">
@@ -7219,7 +7219,7 @@
       </c>
       <c r="H75" s="27" t="inlineStr">
         <is>
-          <t>Tense, focused.</t>
+          <t>Grudging, a bit flirty.</t>
         </is>
       </c>
       <c r="I75" s="27" t="n"/>
@@ -7231,12 +7231,12 @@
       </c>
       <c r="B76" s="24" t="inlineStr">
         <is>
-          <t>marina_chat_02</t>
+          <t>marina_chat_04</t>
         </is>
       </c>
       <c r="C76" s="23" t="inlineStr">
         <is>
-          <t>marina_chat_02.wav</t>
+          <t>marina_chat_04.wav</t>
         </is>
       </c>
       <c r="D76" s="24" t="inlineStr">
@@ -7251,7 +7251,7 @@
       </c>
       <c r="F76" s="25" t="inlineStr">
         <is>
-          <t>You're getting good at this. It's annoying.</t>
+          <t>If anyone asks, we're friends. Who swim. At night.</t>
         </is>
       </c>
       <c r="G76" s="24" t="inlineStr">
@@ -7261,7 +7261,7 @@
       </c>
       <c r="H76" s="24" t="inlineStr">
         <is>
-          <t>Grudging, a bit flirty.</t>
+          <t>Fast, flustered.</t>
         </is>
       </c>
       <c r="I76" s="24" t="n"/>
@@ -7273,12 +7273,12 @@
       </c>
       <c r="B77" s="27" t="inlineStr">
         <is>
-          <t>marina_chat_03</t>
+          <t>marina_chat_05</t>
         </is>
       </c>
       <c r="C77" s="26" t="inlineStr">
         <is>
-          <t>marina_chat_03.wav</t>
+          <t>marina_chat_05.wav</t>
         </is>
       </c>
       <c r="D77" s="27" t="inlineStr">
@@ -7293,7 +7293,7 @@
       </c>
       <c r="F77" s="28" t="inlineStr">
         <is>
-          <t>Gran says hello. Gran says a lot of things.</t>
+          <t>Board, lifeguard. Not me.</t>
         </is>
       </c>
       <c r="G77" s="27" t="inlineStr">
@@ -7303,7 +7303,7 @@
       </c>
       <c r="H77" s="27" t="inlineStr">
         <is>
-          <t>Long-suffering.</t>
+          <t>Teasing; caught you looking.</t>
         </is>
       </c>
       <c r="I77" s="27" t="n"/>
@@ -7315,12 +7315,12 @@
       </c>
       <c r="B78" s="24" t="inlineStr">
         <is>
-          <t>marina_chat_04</t>
+          <t>marina_chat_07</t>
         </is>
       </c>
       <c r="C78" s="23" t="inlineStr">
         <is>
-          <t>marina_chat_04.wav</t>
+          <t>marina_chat_07.wav</t>
         </is>
       </c>
       <c r="D78" s="24" t="inlineStr">
@@ -7335,7 +7335,7 @@
       </c>
       <c r="F78" s="25" t="inlineStr">
         <is>
-          <t>If Nerissa asks, we're friends. Who swim. At night.</t>
+          <t>Mum wants to feed you. Consider yourself warned.</t>
         </is>
       </c>
       <c r="G78" s="24" t="inlineStr">
@@ -7345,7 +7345,7 @@
       </c>
       <c r="H78" s="24" t="inlineStr">
         <is>
-          <t>Fast, flustered.</t>
+          <t>Wry.</t>
         </is>
       </c>
       <c r="I78" s="24" t="n"/>
@@ -7357,12 +7357,12 @@
       </c>
       <c r="B79" s="27" t="inlineStr">
         <is>
-          <t>marina_chat_05</t>
+          <t>marina_chat_08</t>
         </is>
       </c>
       <c r="C79" s="26" t="inlineStr">
         <is>
-          <t>marina_chat_05.wav</t>
+          <t>marina_chat_08.wav</t>
         </is>
       </c>
       <c r="D79" s="27" t="inlineStr">
@@ -7377,7 +7377,7 @@
       </c>
       <c r="F79" s="28" t="inlineStr">
         <is>
-          <t>Board, lifeguard. Not me.</t>
+          <t>Faster. Tide's turning.</t>
         </is>
       </c>
       <c r="G79" s="27" t="inlineStr">
@@ -7387,145 +7387,19 @@
       </c>
       <c r="H79" s="27" t="inlineStr">
         <is>
-          <t>Teasing; caught you looking.</t>
+          <t>Brisk, urgent.</t>
         </is>
       </c>
       <c r="I79" s="27" t="n"/>
       <c r="J79" s="27" t="n"/>
     </row>
-    <row r="80" ht="27" customHeight="1">
-      <c r="A80" s="23" t="n">
-        <v>75</v>
-      </c>
-      <c r="B80" s="24" t="inlineStr">
-        <is>
-          <t>marina_chat_06</t>
-        </is>
-      </c>
-      <c r="C80" s="23" t="inlineStr">
-        <is>
-          <t>marina_chat_06.wav</t>
-        </is>
-      </c>
-      <c r="D80" s="24" t="inlineStr">
-        <is>
-          <t>Puzzle quip: chatter while you play</t>
-        </is>
-      </c>
-      <c r="E80" s="23" t="inlineStr">
-        <is>
-          <t>Short bark, shown as a pop-up while you play.</t>
-        </is>
-      </c>
-      <c r="F80" s="25" t="inlineStr">
-        <is>
-          <t>You still only have one shoe, you know.</t>
-        </is>
-      </c>
-      <c r="G80" s="24" t="inlineStr">
-        <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="H80" s="24" t="inlineStr">
-        <is>
-          <t>Deadpan.</t>
-        </is>
-      </c>
-      <c r="I80" s="24" t="n"/>
-      <c r="J80" s="24" t="n"/>
-    </row>
-    <row r="81" ht="27" customHeight="1">
-      <c r="A81" s="26" t="n">
-        <v>76</v>
-      </c>
-      <c r="B81" s="27" t="inlineStr">
-        <is>
-          <t>marina_chat_07</t>
-        </is>
-      </c>
-      <c r="C81" s="26" t="inlineStr">
-        <is>
-          <t>marina_chat_07.wav</t>
-        </is>
-      </c>
-      <c r="D81" s="27" t="inlineStr">
-        <is>
-          <t>Puzzle quip: chatter while you play</t>
-        </is>
-      </c>
-      <c r="E81" s="26" t="inlineStr">
-        <is>
-          <t>Short bark, shown as a pop-up while you play.</t>
-        </is>
-      </c>
-      <c r="F81" s="28" t="inlineStr">
-        <is>
-          <t>Mum wants to feed you. Consider yourself warned.</t>
-        </is>
-      </c>
-      <c r="G81" s="27" t="inlineStr">
-        <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="H81" s="27" t="inlineStr">
-        <is>
-          <t>Wry.</t>
-        </is>
-      </c>
-      <c r="I81" s="27" t="n"/>
-      <c r="J81" s="27" t="n"/>
-    </row>
-    <row r="82" ht="27" customHeight="1">
-      <c r="A82" s="23" t="n">
-        <v>77</v>
-      </c>
-      <c r="B82" s="24" t="inlineStr">
-        <is>
-          <t>marina_chat_08</t>
-        </is>
-      </c>
-      <c r="C82" s="23" t="inlineStr">
-        <is>
-          <t>marina_chat_08.wav</t>
-        </is>
-      </c>
-      <c r="D82" s="24" t="inlineStr">
-        <is>
-          <t>Puzzle quip: chatter while you play</t>
-        </is>
-      </c>
-      <c r="E82" s="23" t="inlineStr">
-        <is>
-          <t>Short bark, shown as a pop-up while you play.</t>
-        </is>
-      </c>
-      <c r="F82" s="25" t="inlineStr">
-        <is>
-          <t>Faster. Tide's turning.</t>
-        </is>
-      </c>
-      <c r="G82" s="24" t="inlineStr">
-        <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="H82" s="24" t="inlineStr">
-        <is>
-          <t>Brisk, urgent.</t>
-        </is>
-      </c>
-      <c r="I82" s="24" t="n"/>
-      <c r="J82" s="24" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A5:J82"/>
+  <autoFilter ref="A5:J79"/>
   <mergeCells count="1">
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I6:I82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I6:I79" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Hazel's recorded script and 72 voice clips; Whisper check of every clip
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TeVA9WJDfvrL1N6Qe3Kpqx
</commit_message>
<xml_diff>
--- a/docs/voice/Charm_Combo_Voice_Script.xlsx
+++ b/docs/voice/Charm_Combo_Voice_Script.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Marina'!$5:$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Opal'!$A$5:$J$79</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Opal'!$5:$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Hazel'!$A$5:$J$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Hazel'!$A$5:$J$71</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Hazel'!$5:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4815,7 +4815,7 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>That's off the comb's box. So it went in right here.</t>
+          <t>That's off the comb's box. So it went right in there.</t>
         </is>
       </c>
       <c r="G18" s="24" t="inlineStr">
@@ -4852,7 +4852,7 @@
       </c>
       <c r="E19" s="26" t="inlineStr">
         <is>
-          <t>Her previous line: That's off the comb's box. So it went in right here.</t>
+          <t>Her previous line: That's off the comb's box. So it went right in there.</t>
         </is>
       </c>
       <c r="F19" s="28" t="inlineStr">
@@ -6075,7 +6075,7 @@
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>There. Now you can't go anywhere. That's a mermaid thing. It's very old. I just made it up.</t>
+          <t>There. Now you can't go anywhere. It's a mermaid thing. It's very old. I just made it up.</t>
         </is>
       </c>
       <c r="G48" s="24" t="inlineStr">
@@ -10651,7 +10651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J78"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -10790,12 +10790,12 @@
       </c>
       <c r="G6" s="24" t="inlineStr">
         <is>
-          <t>angry</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="H6" s="24" t="inlineStr">
         <is>
-          <t>You're about to cut her tree. Calm, but threatening.</t>
+          <t>Calm.</t>
         </is>
       </c>
       <c r="I6" s="24" t="n"/>
@@ -10827,17 +10827,17 @@
       </c>
       <c r="F7" s="28" t="inlineStr">
         <is>
-          <t>You were aiming just below my heart. That takes forty years or so to heal.</t>
+          <t>You'd have struck just below my heart. It would take... forty years or so to heal.</t>
         </is>
       </c>
       <c r="G7" s="27" t="inlineStr">
         <is>
-          <t>sad</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="H7" s="27" t="inlineStr">
         <is>
-          <t>Calm, not angry, a little sad.</t>
+          <t>Serious.</t>
         </is>
       </c>
       <c r="I7" s="27" t="n"/>
@@ -10864,22 +10864,22 @@
       </c>
       <c r="E8" s="23" t="inlineStr">
         <is>
-          <t>Her previous line: You were aiming just below my heart. That takes forty years or so to heal.</t>
+          <t>Her previous line: You'd have struck just below my heart. It would take... forty years or so to heal.</t>
         </is>
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>Let me guess. Aldous paid you half up front.</t>
+          <t>The miller sent you? He sends someone every spring.</t>
         </is>
       </c>
       <c r="G8" s="24" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>angry</t>
         </is>
       </c>
       <c r="H8" s="24" t="inlineStr">
         <is>
-          <t>Dry, tired more than cross. Aldous the miller sends someone every spring.</t>
+          <t>Annoyed.</t>
         </is>
       </c>
       <c r="I8" s="24" t="n"/>
@@ -10911,7 +10911,7 @@
       </c>
       <c r="F9" s="28" t="inlineStr">
         <is>
-          <t>Oh. You're putting it down. Most of them argue first.</t>
+          <t>Oh, you're putting it down. Most argue first.</t>
         </is>
       </c>
       <c r="G9" s="27" t="inlineStr">
@@ -10921,13 +10921,13 @@
       </c>
       <c r="H9" s="27" t="inlineStr">
         <is>
-          <t>Mildly surprised. A little disarmed.</t>
+          <t>Surprised.</t>
         </is>
       </c>
       <c r="I9" s="27" t="n"/>
       <c r="J9" s="27" t="n"/>
     </row>
-    <row r="10" ht="40.5" customHeight="1">
+    <row r="10" ht="27" customHeight="1">
       <c r="A10" s="23" t="n">
         <v>5</v>
       </c>
@@ -10948,22 +10948,22 @@
       </c>
       <c r="E10" s="23" t="inlineStr">
         <is>
-          <t>Her previous line: Oh. You're putting it down. Most of them argue first.</t>
+          <t>Her previous line: Oh, you're putting it down. Most argue first.</t>
         </is>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
-          <t>The last one argued with the axe still in his hands, so I dropped a beehive on him. I wouldn't do that to you. Your face is too nice to waste on bees.</t>
+          <t>I had to drop a branch on the last guy, but don't worry, your face is too nice.</t>
         </is>
       </c>
       <c r="G10" s="24" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>teasing</t>
         </is>
       </c>
       <c r="H10" s="24" t="inlineStr">
         <is>
-          <t>Bone-dry, perfectly pleasant. The compliment comes out in the same flat tone.</t>
+          <t>Flirting.</t>
         </is>
       </c>
       <c r="I10" s="24" t="n"/>
@@ -10995,7 +10995,7 @@
       </c>
       <c r="F11" s="28" t="inlineStr">
         <is>
-          <t>I know about the wall. My roots go where the water is, and they've never once asked my opinion.</t>
+          <t>I know about the wall. My roots go where the water is. I can't control it.</t>
         </is>
       </c>
       <c r="G11" s="27" t="inlineStr">
@@ -11005,13 +11005,13 @@
       </c>
       <c r="H11" s="27" t="inlineStr">
         <is>
-          <t>Tired. She's had this argument with herself for years.</t>
+          <t>Tired.</t>
         </is>
       </c>
       <c r="I11" s="27" t="n"/>
       <c r="J11" s="27" t="n"/>
     </row>
-    <row r="12" ht="54" customHeight="1">
+    <row r="12" ht="40.5" customHeight="1">
       <c r="A12" s="23" t="n">
         <v>7</v>
       </c>
@@ -11032,28 +11032,28 @@
       </c>
       <c r="E12" s="23" t="inlineStr">
         <is>
-          <t>Her previous line: I know about the wall. My roots go where the water is, and they've never once asked my opinion.</t>
+          <t>Her previous line: I know about the wall. My roots go where the water is. I can't control it.</t>
         </is>
       </c>
       <c r="F12" s="25" t="inlineStr">
         <is>
-          <t>If someone dug him a new channel further out, my roots would follow the water. It would take a season. Nobody's ever offered. It's a lot of digging.</t>
+          <t>If someone dug him a new channel, further out, I could follow it. It would take a season.</t>
         </is>
       </c>
       <c r="G12" s="24" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>happy</t>
         </is>
       </c>
       <c r="H12" s="24" t="inlineStr">
         <is>
-          <t>Plain. A small hope she won't admit to; the last sentence is a hint.</t>
+          <t>Hopeful.</t>
         </is>
       </c>
       <c r="I12" s="24" t="n"/>
       <c r="J12" s="24" t="n"/>
     </row>
-    <row r="13" ht="40.5" customHeight="1">
+    <row r="13" ht="27" customHeight="1">
       <c r="A13" s="26" t="n">
         <v>8</v>
       </c>
@@ -11079,17 +11079,17 @@
       </c>
       <c r="F13" s="28" t="inlineStr">
         <is>
-          <t>By hand? You'll be at it till midsummer. I suppose I'll have to put up with you all spring.</t>
+          <t>All spring, by hand? I guess I'll have to get used to you.</t>
         </is>
       </c>
       <c r="G13" s="27" t="inlineStr">
         <is>
-          <t>surprised</t>
+          <t>happy</t>
         </is>
       </c>
       <c r="H13" s="27" t="inlineStr">
         <is>
-          <t>Slow disbelief, touched. The second sentence pretends to be a complaint.</t>
+          <t>Happy.</t>
         </is>
       </c>
       <c r="I13" s="27" t="n"/>
@@ -11121,17 +11121,17 @@
       </c>
       <c r="F14" s="25" t="inlineStr">
         <is>
-          <t>Start by the alder, the ground's soft there. And roll your sleeves up. For the digging.</t>
+          <t>Now start at the alder and sleeves up.</t>
         </is>
       </c>
       <c r="G14" s="24" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>teasing</t>
         </is>
       </c>
       <c r="H14" s="24" t="inlineStr">
         <is>
-          <t>Practical, then a short pause before the excuse at the end.</t>
+          <t>Flirting.</t>
         </is>
       </c>
       <c r="I14" s="24" t="n"/>
@@ -11163,23 +11163,23 @@
       </c>
       <c r="F15" s="28" t="inlineStr">
         <is>
-          <t>Keep it. Buy yourself a better axe and never use it.</t>
+          <t>Greedy. Oh, so you'll make him pay you to help me? I like that.</t>
         </is>
       </c>
       <c r="G15" s="27" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>happy</t>
         </is>
       </c>
       <c r="H15" s="27" t="inlineStr">
         <is>
-          <t>Dry, amused.</t>
+          <t>Happy.</t>
         </is>
       </c>
       <c r="I15" s="27" t="n"/>
       <c r="J15" s="27" t="n"/>
     </row>
-    <row r="16" ht="27" customHeight="1">
+    <row r="16" ht="40.5" customHeight="1">
       <c r="A16" s="23" t="n">
         <v>11</v>
       </c>
@@ -11200,12 +11200,12 @@
       </c>
       <c r="E16" s="23" t="inlineStr">
         <is>
-          <t>Her previous line: Keep it. Buy yourself a better axe and never use it.</t>
+          <t>Her previous line: Greedy. Oh, so you'll make him pay you to help me? I like that.</t>
         </is>
       </c>
       <c r="F16" s="25" t="inlineStr">
         <is>
-          <t>Start by the alder. If you hit a root, say sorry. It's me, and I'll be listening.</t>
+          <t>Start at the alder. I'll enjoy the view.</t>
         </is>
       </c>
       <c r="G16" s="24" t="inlineStr">
@@ -11215,7 +11215,7 @@
       </c>
       <c r="H16" s="24" t="inlineStr">
         <is>
-          <t>Deadpan. She means the apology.</t>
+          <t>Teasing.</t>
         </is>
       </c>
       <c r="I16" s="24" t="n"/>
@@ -11247,7 +11247,7 @@
       </c>
       <c r="F17" s="28" t="inlineStr">
         <is>
-          <t>That's a lovely trench, if you're planning to bury somebody. For a millrace it's a start.</t>
+          <t>That's a good trench, for a grave.</t>
         </is>
       </c>
       <c r="G17" s="27" t="inlineStr">
@@ -11257,7 +11257,7 @@
       </c>
       <c r="H17" s="27" t="inlineStr">
         <is>
-          <t>Teasing, unhurried.</t>
+          <t>Teasing.</t>
         </is>
       </c>
       <c r="I17" s="27" t="n"/>
@@ -11289,7 +11289,7 @@
       </c>
       <c r="F18" s="25" t="inlineStr">
         <is>
-          <t>Oh. You're warm. Nobody's put a hand on me in years, unless they were measuring where to cut.</t>
+          <t>Oh, you're warm... No one's touched me without an axe in years.</t>
         </is>
       </c>
       <c r="G18" s="24" t="inlineStr">
@@ -11299,7 +11299,7 @@
       </c>
       <c r="H18" s="24" t="inlineStr">
         <is>
-          <t>Surprised, caught off guard.</t>
+          <t>Surprised.</t>
         </is>
       </c>
       <c r="I18" s="24" t="n"/>
@@ -11331,7 +11331,7 @@
       </c>
       <c r="F19" s="28" t="inlineStr">
         <is>
-          <t>Leave it. Bit lower, if you like. The bark's softer.</t>
+          <t>Leave it there a minute. It's been a long time.</t>
         </is>
       </c>
       <c r="G19" s="27" t="inlineStr">
@@ -11341,7 +11341,7 @@
       </c>
       <c r="H19" s="27" t="inlineStr">
         <is>
-          <t>Quiet and low; a little embarrassed she said it.</t>
+          <t>Shy.</t>
         </is>
       </c>
       <c r="I19" s="27" t="n"/>
@@ -11383,7 +11383,7 @@
       </c>
       <c r="H20" s="24" t="inlineStr">
         <is>
-          <t>Matter-of-fact, the sadness well buried.</t>
+          <t>Sad.</t>
         </is>
       </c>
       <c r="I20" s="24" t="n"/>
@@ -11415,17 +11415,17 @@
       </c>
       <c r="F21" s="28" t="inlineStr">
         <is>
-          <t>The badgers visit. They don't talk much, and none of them has ever leaned on me like that.</t>
+          <t>It isn't so bad, but some animals are... Barely tolerable company.</t>
         </is>
       </c>
       <c r="G21" s="27" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="H21" s="27" t="inlineStr">
         <is>
-          <t>Dry joke, then fond.</t>
+          <t>Teasing.</t>
         </is>
       </c>
       <c r="I21" s="27" t="n"/>
@@ -11467,13 +11467,13 @@
       </c>
       <c r="H22" s="24" t="inlineStr">
         <is>
-          <t>Instant, deadpan.</t>
+          <t>Teasing.</t>
         </is>
       </c>
       <c r="I22" s="24" t="n"/>
       <c r="J22" s="24" t="n"/>
     </row>
-    <row r="23" ht="40.5" customHeight="1">
+    <row r="23" ht="27" customHeight="1">
       <c r="A23" s="26" t="n">
         <v>18</v>
       </c>
@@ -11499,7 +11499,7 @@
       </c>
       <c r="F23" s="28" t="inlineStr">
         <is>
-          <t>Come back tomorrow. Bring the shovel, leave the axe, and wear that shirt again.</t>
+          <t>But I'll allow it. Bring the shovel tomorrow though.</t>
         </is>
       </c>
       <c r="G23" s="27" t="inlineStr">
@@ -11509,7 +11509,7 @@
       </c>
       <c r="H23" s="27" t="inlineStr">
         <is>
-          <t>Warm, playful; the last part comes quickly, before she can take it back.</t>
+          <t>Happy.</t>
         </is>
       </c>
       <c r="I23" s="27" t="n"/>
@@ -11541,7 +11541,7 @@
       </c>
       <c r="F24" s="25" t="inlineStr">
         <is>
-          <t>The ferns say you walked the miller's daughter to the footbridge. That's fine. I'm sure no branch will fall on her. Fairly sure.</t>
+          <t>The ferns tell me you were talking to the miller's daughter. I'm not jealous. But I might drop a branch near her, that's all.</t>
         </is>
       </c>
       <c r="G24" s="24" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="H24" s="24" t="inlineStr">
         <is>
-          <t>Calm and pleasant, and jealous. The threat is polite.</t>
+          <t>Jealous.</t>
         </is>
       </c>
       <c r="I24" s="24" t="n"/>
@@ -11583,17 +11583,17 @@
       </c>
       <c r="F25" s="28" t="inlineStr">
         <is>
-          <t>Her father came by too. You've got till the end of the month. Then he hires someone with a saw.</t>
+          <t>Her father came by this morning. He'll give you until the end of the month. Then he hires someone with a saw.</t>
         </is>
       </c>
       <c r="G25" s="27" t="inlineStr">
         <is>
-          <t>sad</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="H25" s="27" t="inlineStr">
         <is>
-          <t>Calm on the surface; worry underneath.</t>
+          <t>Serious.</t>
         </is>
       </c>
       <c r="I25" s="27" t="n"/>
@@ -11620,22 +11620,22 @@
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
-          <t>Her previous line: Her father came by too. You've got till the end of the month. Then he hires someone with a saw.</t>
+          <t>Her previous line: Her father came by this morning. He'll give you until the end of the month. Then he hires someone with a saw.</t>
         </is>
       </c>
       <c r="F26" s="25" t="inlineStr">
         <is>
-          <t>So dig faster. I've started making plans for summer, and you're in most of them.</t>
+          <t>Dig faster. I'd like to see another spring.</t>
         </is>
       </c>
       <c r="G26" s="24" t="inlineStr">
         <is>
-          <t>shy</t>
+          <t>sad</t>
         </is>
       </c>
       <c r="H26" s="24" t="inlineStr">
         <is>
-          <t>Light on top, real fear underneath; the second half is softer.</t>
+          <t>Scared.</t>
         </is>
       </c>
       <c r="I26" s="24" t="n"/>
@@ -11667,23 +11667,23 @@
       </c>
       <c r="F27" s="28" t="inlineStr">
         <is>
-          <t>I know. The ferns mentioned that too.</t>
+          <t>I know. You were still gone forty minutes, not that I was counting.</t>
         </is>
       </c>
       <c r="G27" s="27" t="inlineStr">
         <is>
-          <t>shy</t>
+          <t>angry</t>
         </is>
       </c>
       <c r="H27" s="27" t="inlineStr">
         <is>
-          <t>Soft, caught out.</t>
+          <t>Jealous.</t>
         </is>
       </c>
       <c r="I27" s="27" t="n"/>
       <c r="J27" s="27" t="n"/>
     </row>
-    <row r="28" ht="27" customHeight="1">
+    <row r="28" ht="40.5" customHeight="1">
       <c r="A28" s="23" t="n">
         <v>23</v>
       </c>
@@ -11704,22 +11704,22 @@
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
-          <t>Her previous line: I know. The ferns mentioned that too.</t>
+          <t>Her previous line: I know. You were still gone forty minutes, not that I was counting.</t>
         </is>
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>Eat your lunch. She makes good bread, apparently. Nobody's ever walked me to a footbridge.</t>
+          <t>Eat your lunch. I'm sure her bread is very good. I wouldn't know.</t>
         </is>
       </c>
       <c r="G28" s="24" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>angry</t>
         </is>
       </c>
       <c r="H28" s="24" t="inlineStr">
         <is>
-          <t>A tiny bit petty, mostly wistful.</t>
+          <t>Jealous.</t>
         </is>
       </c>
       <c r="I28" s="24" t="n"/>
@@ -11756,12 +11756,12 @@
       </c>
       <c r="G29" s="27" t="inlineStr">
         <is>
-          <t>angry</t>
+          <t>shy</t>
         </is>
       </c>
       <c r="H29" s="27" t="inlineStr">
         <is>
-          <t>Clipped, flustered.</t>
+          <t>Flustered.</t>
         </is>
       </c>
       <c r="I29" s="27" t="n"/>
@@ -11793,7 +11793,7 @@
       </c>
       <c r="F30" s="25" t="inlineStr">
         <is>
-          <t>Dig your trench. And stop looking at my leaves.</t>
+          <t>Dig your trench. Sleeves up!</t>
         </is>
       </c>
       <c r="G30" s="24" t="inlineStr">
@@ -11803,7 +11803,7 @@
       </c>
       <c r="H30" s="24" t="inlineStr">
         <is>
-          <t>Mortified, very dignified about it.</t>
+          <t>Flustered.</t>
         </is>
       </c>
       <c r="I30" s="24" t="n"/>
@@ -11835,7 +11835,7 @@
       </c>
       <c r="F31" s="28" t="inlineStr">
         <is>
-          <t>It's fine. It's the roots letting go of the old wall. They've held it forty years. They're making a fuss.</t>
+          <t>It's fine. It's just roots. They have to let go of the old wall even if it hurts.</t>
         </is>
       </c>
       <c r="G31" s="27" t="inlineStr">
@@ -11845,7 +11845,7 @@
       </c>
       <c r="H31" s="27" t="inlineStr">
         <is>
-          <t>Strained. Trying to sound calm and not quite managing.</t>
+          <t>Sad.</t>
         </is>
       </c>
       <c r="I31" s="27" t="n"/>
@@ -11877,7 +11877,7 @@
       </c>
       <c r="F32" s="25" t="inlineStr">
         <is>
-          <t>You didn't have to stay. You're soaked. You'll get ill, and then I'll have to look after you, and I've no idea how.</t>
+          <t>You're shaking. Come in closer, there's a hollow in the trunk that fits you.</t>
         </is>
       </c>
       <c r="G32" s="24" t="inlineStr">
@@ -11887,13 +11887,13 @@
       </c>
       <c r="H32" s="24" t="inlineStr">
         <is>
-          <t>Gruff, grateful underneath.</t>
+          <t>Caring.</t>
         </is>
       </c>
       <c r="I32" s="24" t="n"/>
       <c r="J32" s="24" t="n"/>
     </row>
-    <row r="33" ht="54" customHeight="1">
+    <row r="33" ht="40.5" customHeight="1">
       <c r="A33" s="26" t="n">
         <v>28</v>
       </c>
@@ -11914,12 +11914,12 @@
       </c>
       <c r="E33" s="26" t="inlineStr">
         <is>
-          <t>Her previous line: You didn't have to stay. You're soaked. You'll get ill, and then I'll have to look after you, and I've no idea how.</t>
+          <t>Her previous line: You're shaking. Come in closer, there's a hollow in the trunk that fits you.</t>
         </is>
       </c>
       <c r="F33" s="28" t="inlineStr">
         <is>
-          <t>Talk to me. About anything. What did you have for breakfast?</t>
+          <t>Talk to me. About anything. Your voice helps me get through it.</t>
         </is>
       </c>
       <c r="G33" s="27" t="inlineStr">
@@ -11929,7 +11929,7 @@
       </c>
       <c r="H33" s="27" t="inlineStr">
         <is>
-          <t>Small, strained; asking for help is hard for her, so she makes it about breakfast.</t>
+          <t>Scared.</t>
         </is>
       </c>
       <c r="I33" s="27" t="n"/>
@@ -11971,7 +11971,7 @@
       </c>
       <c r="H34" s="24" t="inlineStr">
         <is>
-          <t>Drifting into a memory; fond, a little wry.</t>
+          <t>Happy.</t>
         </is>
       </c>
       <c r="I34" s="24" t="n"/>
@@ -12003,7 +12003,7 @@
       </c>
       <c r="F35" s="28" t="inlineStr">
         <is>
-          <t>You're still warm. I'll keep you.</t>
+          <t>You're still warm. Good.</t>
         </is>
       </c>
       <c r="G35" s="27" t="inlineStr">
@@ -12013,7 +12013,7 @@
       </c>
       <c r="H35" s="27" t="inlineStr">
         <is>
-          <t>Barely a murmur, to herself as much as to you.</t>
+          <t>Shy.</t>
         </is>
       </c>
       <c r="I35" s="27" t="n"/>
@@ -12050,12 +12050,12 @@
       </c>
       <c r="G36" s="24" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="H36" s="24" t="inlineStr">
         <is>
-          <t>Perking up, wicked.</t>
+          <t>Teasing.</t>
         </is>
       </c>
       <c r="I36" s="24" t="n"/>
@@ -12097,7 +12097,7 @@
       </c>
       <c r="H37" s="27" t="inlineStr">
         <is>
-          <t>Laughing through the pain.</t>
+          <t>Laughing.</t>
         </is>
       </c>
       <c r="I37" s="27" t="n"/>
@@ -12129,17 +12129,17 @@
       </c>
       <c r="F38" s="25" t="inlineStr">
         <is>
-          <t>Forty springs he's sent people with axes. That's the first time he's ever touched me.</t>
+          <t>He's never done that. Forty springs, and he's never once done that.</t>
         </is>
       </c>
       <c r="G38" s="24" t="inlineStr">
         <is>
-          <t>surprised</t>
+          <t>happy</t>
         </is>
       </c>
       <c r="H38" s="24" t="inlineStr">
         <is>
-          <t>Quietly moved. Almost a whisper.</t>
+          <t>Happy.</t>
         </is>
       </c>
       <c r="I38" s="24" t="n"/>
@@ -12171,7 +12171,7 @@
       </c>
       <c r="F39" s="28" t="inlineStr">
         <is>
-          <t>I can go as far as my roots do. Thanks to someone, that's quite far now. Far enough to follow you home, if I felt like it.</t>
+          <t>I can walk as far as my roots go. They go a long way now. Thanks to someone.</t>
         </is>
       </c>
       <c r="G39" s="27" t="inlineStr">
@@ -12181,13 +12181,13 @@
       </c>
       <c r="H39" s="27" t="inlineStr">
         <is>
-          <t>Shy and warm; won't say your name. The last part is a test.</t>
+          <t>Shy.</t>
         </is>
       </c>
       <c r="I39" s="27" t="n"/>
       <c r="J39" s="27" t="n"/>
     </row>
-    <row r="40" ht="54" customHeight="1">
+    <row r="40" ht="40.5" customHeight="1">
       <c r="A40" s="23" t="n">
         <v>35</v>
       </c>
@@ -12208,12 +12208,12 @@
       </c>
       <c r="E40" s="23" t="inlineStr">
         <is>
-          <t>Her previous line: I can go as far as my roots do. Thanks to someone, that's quite far now. Far enough to follow you home, if I felt like it.</t>
+          <t>Her previous line: I can walk as far as my roots go. They go a long way now. Thanks to someone.</t>
         </is>
       </c>
       <c r="F40" s="25" t="inlineStr">
         <is>
-          <t>The moss on the east side is softer than it looks. I've been meaning to mention that for about a week.</t>
+          <t>The moss on the east side is softer than it looks.</t>
         </is>
       </c>
       <c r="G40" s="24" t="inlineStr">
@@ -12223,13 +12223,13 @@
       </c>
       <c r="H40" s="24" t="inlineStr">
         <is>
-          <t>Low and slow. An invitation she's pretending is a fact about moss.</t>
+          <t>Flirting.</t>
         </is>
       </c>
       <c r="I40" s="24" t="n"/>
       <c r="J40" s="24" t="n"/>
     </row>
-    <row r="41" ht="54" customHeight="1">
+    <row r="41" ht="27" customHeight="1">
       <c r="A41" s="26" t="n">
         <v>36</v>
       </c>
@@ -12250,22 +12250,22 @@
       </c>
       <c r="E41" s="26" t="inlineStr">
         <is>
-          <t>Her previous line: The moss on the east side is softer than it looks. I've been meaning to mention that for about a week.</t>
+          <t>Her previous line: The moss on the east side is softer than it looks.</t>
         </is>
       </c>
       <c r="F41" s="28" t="inlineStr">
         <is>
-          <t>Stay tonight. I'll keep the rain off. I'm not promising anything else.</t>
+          <t>Stay tonight. I'll keep the rain off.</t>
         </is>
       </c>
       <c r="G41" s="27" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>teasing</t>
         </is>
       </c>
       <c r="H41" s="27" t="inlineStr">
         <is>
-          <t>Warm, certain, a little wicked at the end.</t>
+          <t>Flirting.</t>
         </is>
       </c>
       <c r="I41" s="27" t="n"/>
@@ -12297,17 +12297,17 @@
       </c>
       <c r="F42" s="25" t="inlineStr">
         <is>
-          <t>Two hundred years people have walked past this tree. Not one of them ever lay down under it. Shift over, you're on a root.</t>
+          <t>Two hundred springs I've watched people walk past this tree. Not one of them ever lay down under it.</t>
         </is>
       </c>
       <c r="G42" s="24" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>surprised</t>
         </is>
       </c>
       <c r="H42" s="24" t="inlineStr">
         <is>
-          <t>Slow and calm, quietly amazed, then practical.</t>
+          <t>Surprised.</t>
         </is>
       </c>
       <c r="I42" s="24" t="n"/>
@@ -12334,22 +12334,22 @@
       </c>
       <c r="E43" s="26" t="inlineStr">
         <is>
-          <t>Her previous line: Two hundred years people have walked past this tree. Not one of them ever lay down under it. Shift over, you're on a root.</t>
+          <t>Her previous line: Two hundred springs I've watched people walk past this tree. Not one of them ever lay down under it.</t>
         </is>
       </c>
       <c r="F43" s="28" t="inlineStr">
         <is>
-          <t>The badgers are watching. I told them to go away. Nobody in this grove listens to me.</t>
+          <t>The animals are watching. I told them to go away. Nobody in this grove listens to me.</t>
         </is>
       </c>
       <c r="G43" s="27" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>shy</t>
         </is>
       </c>
       <c r="H43" s="27" t="inlineStr">
         <is>
-          <t>Bone-dry, a little shy under it.</t>
+          <t>Shy.</t>
         </is>
       </c>
       <c r="I43" s="27" t="n"/>
@@ -12386,12 +12386,12 @@
       </c>
       <c r="G44" s="24" t="inlineStr">
         <is>
-          <t>shy</t>
+          <t>teasing</t>
         </is>
       </c>
       <c r="H44" s="24" t="inlineStr">
         <is>
-          <t>Soft, almost accusing. Fond.</t>
+          <t>Flirting.</t>
         </is>
       </c>
       <c r="I44" s="24" t="n"/>
@@ -12433,7 +12433,7 @@
       </c>
       <c r="H45" s="27" t="inlineStr">
         <is>
-          <t>Deadpan joke; nervous underneath.</t>
+          <t>Nervous.</t>
         </is>
       </c>
       <c r="I45" s="27" t="n"/>
@@ -12465,17 +12465,17 @@
       </c>
       <c r="F46" s="25" t="inlineStr">
         <is>
-          <t>Slowly. I've had two hundred years of nothing happening. I'd like this to take a while.</t>
+          <t>Slowly. I've got all the time in the world, and I'd like to spend some of it on this.</t>
         </is>
       </c>
       <c r="G46" s="24" t="inlineStr">
         <is>
-          <t>shy</t>
+          <t>teasing</t>
         </is>
       </c>
       <c r="H46" s="24" t="inlineStr">
         <is>
-          <t>Calm, warm, certain.</t>
+          <t>Flirting.</t>
         </is>
       </c>
       <c r="I46" s="24" t="n"/>
@@ -12507,7 +12507,7 @@
       </c>
       <c r="F47" s="28" t="inlineStr">
         <is>
-          <t>Don't look at the leaves. They're being ridiculous.</t>
+          <t>Don't... look at me like that.</t>
         </is>
       </c>
       <c r="G47" s="27" t="inlineStr">
@@ -12517,39 +12517,39 @@
       </c>
       <c r="H47" s="27" t="inlineStr">
         <is>
-          <t>Embarrassed. She can't control them and she knows you know.</t>
+          <t>Flustered.</t>
         </is>
       </c>
       <c r="I47" s="27" t="n"/>
       <c r="J47" s="27" t="n"/>
     </row>
-    <row r="48" ht="27" customHeight="1">
+    <row r="48" ht="54" customHeight="1">
       <c r="A48" s="23" t="n">
         <v>43</v>
       </c>
       <c r="B48" s="24" t="inlineStr">
         <is>
-          <t>hazel_night_22</t>
+          <t>hazel_end_01</t>
         </is>
       </c>
       <c r="C48" s="23" t="inlineStr">
         <is>
-          <t>hazel_night_22.wav</t>
-        </is>
-      </c>
-      <c r="D48" s="24" t="inlineStr">
-        <is>
-          <t>Her night scene (full-screen CG)</t>
+          <t>hazel_end_01.wav</t>
+        </is>
+      </c>
+      <c r="D48" s="25" t="inlineStr">
+        <is>
+          <t>Her ending: the morning after</t>
         </is>
       </c>
       <c r="E48" s="23" t="inlineStr">
         <is>
-          <t>Her previous line: Don't look at the leaves. They're being ridiculous.</t>
+          <t>Morning in the grove. There's blossom on the east side of the tree that wasn't there last night. Hazels flower in February. It's May.</t>
         </is>
       </c>
       <c r="F48" s="25" t="inlineStr">
         <is>
-          <t>And don't tell the ferns. They'll want details.</t>
+          <t>Two hundred years, and nobody told me a spirit could feel like that. I'd like it noted that I'm saying this very calmly.</t>
         </is>
       </c>
       <c r="G48" s="24" t="inlineStr">
@@ -12559,108 +12559,108 @@
       </c>
       <c r="H48" s="24" t="inlineStr">
         <is>
-          <t>Hushed, smiling.</t>
+          <t>Happy.</t>
         </is>
       </c>
       <c r="I48" s="24" t="n"/>
       <c r="J48" s="24" t="n"/>
     </row>
-    <row r="49" ht="27" customHeight="1">
+    <row r="49" ht="54" customHeight="1">
       <c r="A49" s="26" t="n">
         <v>44</v>
       </c>
       <c r="B49" s="27" t="inlineStr">
         <is>
-          <t>hazel_night_23</t>
+          <t>hazel_end_02</t>
         </is>
       </c>
       <c r="C49" s="26" t="inlineStr">
         <is>
-          <t>hazel_night_23.wav</t>
+          <t>hazel_end_02.wav</t>
         </is>
       </c>
       <c r="D49" s="27" t="inlineStr">
         <is>
-          <t>Her night scene (full-screen CG)</t>
+          <t>Her ending: the morning after</t>
         </is>
       </c>
       <c r="E49" s="26" t="inlineStr">
         <is>
-          <t>Her previous line: And don't tell the ferns. They'll want details.</t>
+          <t>Her previous line: Two hundred years, and nobody told me a spirit could feel like that. I'd like it noted that I'm saying this very calmly.</t>
         </is>
       </c>
       <c r="F49" s="28" t="inlineStr">
         <is>
-          <t>Sleep. I'll wake you if the miller comes. I might not.</t>
+          <t>Don't look at them. They're not for you. They're seasonal.</t>
         </is>
       </c>
       <c r="G49" s="27" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>shy</t>
         </is>
       </c>
       <c r="H49" s="27" t="inlineStr">
         <is>
-          <t>Warm and drowsy, a little wicked.</t>
+          <t>Flustered.</t>
         </is>
       </c>
       <c r="I49" s="27" t="n"/>
       <c r="J49" s="27" t="n"/>
     </row>
-    <row r="50" ht="54" customHeight="1">
+    <row r="50" ht="40.5" customHeight="1">
       <c r="A50" s="23" t="n">
         <v>45</v>
       </c>
       <c r="B50" s="24" t="inlineStr">
         <is>
-          <t>hazel_end_01</t>
+          <t>hazel_end_03</t>
         </is>
       </c>
       <c r="C50" s="23" t="inlineStr">
         <is>
-          <t>hazel_end_01.wav</t>
-        </is>
-      </c>
-      <c r="D50" s="25" t="inlineStr">
+          <t>hazel_end_03.wav</t>
+        </is>
+      </c>
+      <c r="D50" s="24" t="inlineStr">
         <is>
           <t>Her ending: the morning after</t>
         </is>
       </c>
       <c r="E50" s="23" t="inlineStr">
         <is>
-          <t>Morning in the grove. There's blossom on the east side of the tree that wasn't there last night. Hazels flower in February. It's May.</t>
+          <t>Her previous line: Don't look at them. They're not for you. They're seasonal.</t>
         </is>
       </c>
       <c r="F50" s="25" t="inlineStr">
         <is>
-          <t>Two hundred years, and nobody told me it could feel like that. I'd like it noted that I'm saying this very calmly.</t>
+          <t>Fine. They're for you. I haven't flowered out of season since before the mill was built. The animals are going to talk.</t>
         </is>
       </c>
       <c r="G50" s="24" t="inlineStr">
         <is>
-          <t>shy</t>
+          <t>happy</t>
         </is>
       </c>
       <c r="H50" s="24" t="inlineStr">
         <is>
-          <t>Calm voice, completely undone underneath.</t>
+          <t>Happy.</t>
         </is>
       </c>
       <c r="I50" s="24" t="n"/>
       <c r="J50" s="24" t="n"/>
     </row>
-    <row r="51" ht="54" customHeight="1">
+    <row r="51" ht="40.5" customHeight="1">
       <c r="A51" s="26" t="n">
         <v>46</v>
       </c>
       <c r="B51" s="27" t="inlineStr">
         <is>
-          <t>hazel_end_02</t>
+          <t>hazel_end_04</t>
         </is>
       </c>
       <c r="C51" s="26" t="inlineStr">
         <is>
-          <t>hazel_end_02.wav</t>
+          <t>hazel_end_04.wav</t>
         </is>
       </c>
       <c r="D51" s="27" t="inlineStr">
@@ -12670,22 +12670,22 @@
       </c>
       <c r="E51" s="26" t="inlineStr">
         <is>
-          <t>Her previous line: Two hundred years, and nobody told me it could feel like that. I'd like it noted that I'm saying this very calmly.</t>
+          <t>She shows you which branches you can sit on and which ones she's ticklish about. The second list is long.</t>
         </is>
       </c>
       <c r="F51" s="28" t="inlineStr">
         <is>
-          <t>Don't look at them. They're not for you. They're seasonal.</t>
+          <t>That one's fine. That one's fine. Not that one. I mean it. Don't.</t>
         </is>
       </c>
       <c r="G51" s="27" t="inlineStr">
         <is>
-          <t>shy</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="H51" s="27" t="inlineStr">
         <is>
-          <t>Flustered and a terrible liar, deadpan anyway.</t>
+          <t>Teasing.</t>
         </is>
       </c>
       <c r="I51" s="27" t="n"/>
@@ -12697,12 +12697,12 @@
       </c>
       <c r="B52" s="24" t="inlineStr">
         <is>
-          <t>hazel_end_03</t>
+          <t>hazel_end_05</t>
         </is>
       </c>
       <c r="C52" s="23" t="inlineStr">
         <is>
-          <t>hazel_end_03.wav</t>
+          <t>hazel_end_05.wav</t>
         </is>
       </c>
       <c r="D52" s="24" t="inlineStr">
@@ -12712,54 +12712,54 @@
       </c>
       <c r="E52" s="23" t="inlineStr">
         <is>
-          <t>Her previous line: Don't look at them. They're not for you. They're seasonal.</t>
+          <t>Her previous line: That one's fine. That one's fine. Not that one. I mean it. Don't.</t>
         </is>
       </c>
       <c r="F52" s="25" t="inlineStr">
         <is>
-          <t>Fine. They're for you. I haven't flowered out of season since before the mill was built. People are going to talk.</t>
+          <t>Plant something near me. So there's something of yours here when you're not.</t>
         </is>
       </c>
       <c r="G52" s="24" t="inlineStr">
         <is>
-          <t>happy</t>
+          <t>shy</t>
         </is>
       </c>
       <c r="H52" s="24" t="inlineStr">
         <is>
-          <t>Giving in; fond and a bit exasperated with herself.</t>
+          <t>Shy.</t>
         </is>
       </c>
       <c r="I52" s="24" t="n"/>
       <c r="J52" s="24" t="n"/>
     </row>
-    <row r="53" ht="40.5" customHeight="1">
+    <row r="53" ht="54" customHeight="1">
       <c r="A53" s="26" t="n">
         <v>48</v>
       </c>
       <c r="B53" s="27" t="inlineStr">
         <is>
-          <t>hazel_end_04</t>
+          <t>hazel_gift_01</t>
         </is>
       </c>
       <c r="C53" s="26" t="inlineStr">
         <is>
-          <t>hazel_end_04.wav</t>
-        </is>
-      </c>
-      <c r="D53" s="27" t="inlineStr">
-        <is>
-          <t>Her ending: the morning after</t>
+          <t>hazel_gift_01.wav</t>
+        </is>
+      </c>
+      <c r="D53" s="28" t="inlineStr">
+        <is>
+          <t>Gift scene (Brass Pocket Sundial)</t>
         </is>
       </c>
       <c r="E53" s="26" t="inlineStr">
         <is>
-          <t>She shows you which branches you can sit on and which ones she's ticklish about. The second list is long.</t>
+          <t>She makes you hold it up in the one patch of sun that gets through her leaves, and watches the shadow for a long time.</t>
         </is>
       </c>
       <c r="F53" s="28" t="inlineStr">
         <is>
-          <t>That one's fine. That one's fine. Not that one. I mean it. Don't.</t>
+          <t>A clock that only works when the sun's out.</t>
         </is>
       </c>
       <c r="G53" s="27" t="inlineStr">
@@ -12769,7 +12769,7 @@
       </c>
       <c r="H53" s="27" t="inlineStr">
         <is>
-          <t>Escalating warning, trying not to laugh.</t>
+          <t>Happy.</t>
         </is>
       </c>
       <c r="I53" s="27" t="n"/>
@@ -12781,27 +12781,27 @@
       </c>
       <c r="B54" s="24" t="inlineStr">
         <is>
-          <t>hazel_end_05</t>
+          <t>hazel_gift_02</t>
         </is>
       </c>
       <c r="C54" s="23" t="inlineStr">
         <is>
-          <t>hazel_end_05.wav</t>
+          <t>hazel_gift_02.wav</t>
         </is>
       </c>
       <c r="D54" s="24" t="inlineStr">
         <is>
-          <t>Her ending: the morning after</t>
+          <t>Gift scene (Brass Pocket Sundial)</t>
         </is>
       </c>
       <c r="E54" s="23" t="inlineStr">
         <is>
-          <t>Her previous line: That one's fine. That one's fine. Not that one. I mean it. Don't.</t>
+          <t>The green at the tips of her hair goes a shade darker. She notices, and decides not to mention it.</t>
         </is>
       </c>
       <c r="F54" s="25" t="inlineStr">
         <is>
-          <t>Plant something near me. Something that needs watering every day, so you've got a reason to come by.</t>
+          <t>I'll keep it on a low branch where I can see it. No, I won't use it to count time until our next meeting.</t>
         </is>
       </c>
       <c r="G54" s="24" t="inlineStr">
@@ -12811,49 +12811,49 @@
       </c>
       <c r="H54" s="24" t="inlineStr">
         <is>
-          <t>Simple, a little shy; she's thought about it.</t>
+          <t>Shy.</t>
         </is>
       </c>
       <c r="I54" s="24" t="n"/>
       <c r="J54" s="24" t="n"/>
     </row>
-    <row r="55" ht="54" customHeight="1">
+    <row r="55" ht="27" customHeight="1">
       <c r="A55" s="26" t="n">
         <v>50</v>
       </c>
       <c r="B55" s="27" t="inlineStr">
         <is>
-          <t>hazel_end_06</t>
+          <t>hazel_fav_01</t>
         </is>
       </c>
       <c r="C55" s="26" t="inlineStr">
         <is>
-          <t>hazel_end_06.wav</t>
-        </is>
-      </c>
-      <c r="D55" s="27" t="inlineStr">
-        <is>
-          <t>Her ending: the morning after</t>
+          <t>hazel_fav_01.wav</t>
+        </is>
+      </c>
+      <c r="D55" s="28" t="inlineStr">
+        <is>
+          <t>Puzzle quip: you matched her favourite gem</t>
         </is>
       </c>
       <c r="E55" s="26" t="inlineStr">
         <is>
-          <t>Her previous line: Plant something near me. Something that needs watering every day, so you've got a reason to come by.</t>
+          <t>Short bark, shown as a pop-up while you play.</t>
         </is>
       </c>
       <c r="F55" s="28" t="inlineStr">
         <is>
-          <t>Go on, then. What are you planting? It'll outlast both of us. Well. It'll outlast you.</t>
+          <t>Petals. Good. Those I understand.</t>
         </is>
       </c>
       <c r="G55" s="27" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>happy</t>
         </is>
       </c>
       <c r="H55" s="27" t="inlineStr">
         <is>
-          <t>Gentle, dry correction at the end.</t>
+          <t>Happy.</t>
         </is>
       </c>
       <c r="I55" s="27" t="n"/>
@@ -12865,121 +12865,121 @@
       </c>
       <c r="B56" s="24" t="inlineStr">
         <is>
-          <t>hazel_end_07</t>
+          <t>hazel_fav_02</t>
         </is>
       </c>
       <c r="C56" s="23" t="inlineStr">
         <is>
-          <t>hazel_end_07.wav</t>
+          <t>hazel_fav_02.wav</t>
         </is>
       </c>
       <c r="D56" s="24" t="inlineStr">
         <is>
-          <t>Her ending: the morning after</t>
+          <t>Puzzle quip: you matched her favourite gem</t>
         </is>
       </c>
       <c r="E56" s="23" t="inlineStr">
         <is>
-          <t>You say another hazel, so she isn't the only one.</t>
+          <t>Short bark, shown as a pop-up while you play.</t>
         </is>
       </c>
       <c r="F56" s="25" t="inlineStr">
         <is>
-          <t>A neighbour. I've never had a neighbour.</t>
+          <t>Mm. That one smells like April.</t>
         </is>
       </c>
       <c r="G56" s="24" t="inlineStr">
         <is>
-          <t>shy</t>
+          <t>happy</t>
         </is>
       </c>
       <c r="H56" s="24" t="inlineStr">
         <is>
-          <t>Quiet wonder.</t>
+          <t>Happy.</t>
         </is>
       </c>
       <c r="I56" s="24" t="n"/>
       <c r="J56" s="24" t="n"/>
     </row>
-    <row r="57" ht="54" customHeight="1">
+    <row r="57" ht="27" customHeight="1">
       <c r="A57" s="26" t="n">
         <v>52</v>
       </c>
       <c r="B57" s="27" t="inlineStr">
         <is>
-          <t>hazel_gift_01</t>
+          <t>hazel_fav_03</t>
         </is>
       </c>
       <c r="C57" s="26" t="inlineStr">
         <is>
-          <t>hazel_gift_01.wav</t>
-        </is>
-      </c>
-      <c r="D57" s="28" t="inlineStr">
-        <is>
-          <t>Gift scene (Brass Pocket Sundial)</t>
+          <t>hazel_fav_03.wav</t>
+        </is>
+      </c>
+      <c r="D57" s="27" t="inlineStr">
+        <is>
+          <t>Puzzle quip: you matched her favourite gem</t>
         </is>
       </c>
       <c r="E57" s="26" t="inlineStr">
         <is>
-          <t>She makes you hold it up in the one patch of sun that gets through her leaves, and watches the shadow for a long time.</t>
+          <t>Short bark, shown as a pop-up while you play.</t>
         </is>
       </c>
       <c r="F57" s="28" t="inlineStr">
         <is>
-          <t>A clock that only works when the sun's out. Someone finally made one that keeps sensible hours.</t>
+          <t>Gently. Like that.</t>
         </is>
       </c>
       <c r="G57" s="27" t="inlineStr">
         <is>
-          <t>surprised</t>
+          <t>teasing</t>
         </is>
       </c>
       <c r="H57" s="27" t="inlineStr">
         <is>
-          <t>Delighted, dry. A rare open smile in the voice.</t>
+          <t>Flirting.</t>
         </is>
       </c>
       <c r="I57" s="27" t="n"/>
       <c r="J57" s="27" t="n"/>
     </row>
-    <row r="58" ht="40.5" customHeight="1">
+    <row r="58" ht="27" customHeight="1">
       <c r="A58" s="23" t="n">
         <v>53</v>
       </c>
       <c r="B58" s="24" t="inlineStr">
         <is>
-          <t>hazel_gift_02</t>
+          <t>hazel_fav_04</t>
         </is>
       </c>
       <c r="C58" s="23" t="inlineStr">
         <is>
-          <t>hazel_gift_02.wav</t>
+          <t>hazel_fav_04.wav</t>
         </is>
       </c>
       <c r="D58" s="24" t="inlineStr">
         <is>
-          <t>Gift scene (Brass Pocket Sundial)</t>
+          <t>Puzzle quip: you matched her favourite gem</t>
         </is>
       </c>
       <c r="E58" s="23" t="inlineStr">
         <is>
-          <t>The green at the tips of her hair goes a shade darker. She notices, and decides not to mention it.</t>
+          <t>Short bark, shown as a pop-up while you play.</t>
         </is>
       </c>
       <c r="F58" s="25" t="inlineStr">
         <is>
-          <t>I'll hang it on the low branch. You can see the path from there, which is where you come from. Not that I watch it.</t>
+          <t>You're good with soft things.</t>
         </is>
       </c>
       <c r="G58" s="24" t="inlineStr">
         <is>
-          <t>shy</t>
+          <t>teasing</t>
         </is>
       </c>
       <c r="H58" s="24" t="inlineStr">
         <is>
-          <t>Quiet, shy, saying more than she planned to.</t>
+          <t>Flirting.</t>
         </is>
       </c>
       <c r="I58" s="24" t="n"/>
@@ -12991,15 +12991,15 @@
       </c>
       <c r="B59" s="27" t="inlineStr">
         <is>
-          <t>hazel_fav_01</t>
+          <t>hazel_fav_05</t>
         </is>
       </c>
       <c r="C59" s="26" t="inlineStr">
         <is>
-          <t>hazel_fav_01.wav</t>
-        </is>
-      </c>
-      <c r="D59" s="28" t="inlineStr">
+          <t>hazel_fav_05.wav</t>
+        </is>
+      </c>
+      <c r="D59" s="27" t="inlineStr">
         <is>
           <t>Puzzle quip: you matched her favourite gem</t>
         </is>
@@ -13011,17 +13011,17 @@
       </c>
       <c r="F59" s="28" t="inlineStr">
         <is>
-          <t>Petals. Good. Those I understand.</t>
+          <t>Blossom.</t>
         </is>
       </c>
       <c r="G59" s="27" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>happy</t>
         </is>
       </c>
       <c r="H59" s="27" t="inlineStr">
         <is>
-          <t>Content.</t>
+          <t>Happy.</t>
         </is>
       </c>
       <c r="I59" s="27" t="n"/>
@@ -13033,12 +13033,12 @@
       </c>
       <c r="B60" s="24" t="inlineStr">
         <is>
-          <t>hazel_fav_02</t>
+          <t>hazel_fav_06</t>
         </is>
       </c>
       <c r="C60" s="23" t="inlineStr">
         <is>
-          <t>hazel_fav_02.wav</t>
+          <t>hazel_fav_06.wav</t>
         </is>
       </c>
       <c r="D60" s="24" t="inlineStr">
@@ -13053,17 +13053,17 @@
       </c>
       <c r="F60" s="25" t="inlineStr">
         <is>
-          <t>Mm. That one smells like April.</t>
+          <t>That's lovely. Keep going.</t>
         </is>
       </c>
       <c r="G60" s="24" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>happy</t>
         </is>
       </c>
       <c r="H60" s="24" t="inlineStr">
         <is>
-          <t>Dreamy, slow.</t>
+          <t>Happy.</t>
         </is>
       </c>
       <c r="I60" s="24" t="n"/>
@@ -13075,17 +13075,17 @@
       </c>
       <c r="B61" s="27" t="inlineStr">
         <is>
-          <t>hazel_fav_03</t>
+          <t>hazel_least_01</t>
         </is>
       </c>
       <c r="C61" s="26" t="inlineStr">
         <is>
-          <t>hazel_fav_03.wav</t>
-        </is>
-      </c>
-      <c r="D61" s="27" t="inlineStr">
-        <is>
-          <t>Puzzle quip: you matched her favourite gem</t>
+          <t>hazel_least_01.wav</t>
+        </is>
+      </c>
+      <c r="D61" s="28" t="inlineStr">
+        <is>
+          <t>Puzzle quip: you matched a gem she dislikes</t>
         </is>
       </c>
       <c r="E61" s="26" t="inlineStr">
@@ -13095,17 +13095,17 @@
       </c>
       <c r="F61" s="28" t="inlineStr">
         <is>
-          <t>Gently. Like that.</t>
+          <t>Fire. In a grove. Really?</t>
         </is>
       </c>
       <c r="G61" s="27" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>angry</t>
         </is>
       </c>
       <c r="H61" s="27" t="inlineStr">
         <is>
-          <t>Low, approving.</t>
+          <t>Annoyed.</t>
         </is>
       </c>
       <c r="I61" s="27" t="n"/>
@@ -13117,17 +13117,17 @@
       </c>
       <c r="B62" s="24" t="inlineStr">
         <is>
-          <t>hazel_fav_04</t>
+          <t>hazel_least_02</t>
         </is>
       </c>
       <c r="C62" s="23" t="inlineStr">
         <is>
-          <t>hazel_fav_04.wav</t>
+          <t>hazel_least_02.wav</t>
         </is>
       </c>
       <c r="D62" s="24" t="inlineStr">
         <is>
-          <t>Puzzle quip: you matched her favourite gem</t>
+          <t>Puzzle quip: you matched a gem she dislikes</t>
         </is>
       </c>
       <c r="E62" s="23" t="inlineStr">
@@ -13137,17 +13137,17 @@
       </c>
       <c r="F62" s="25" t="inlineStr">
         <is>
-          <t>You're good with soft things.</t>
+          <t>Put that out.</t>
         </is>
       </c>
       <c r="G62" s="24" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>angry</t>
         </is>
       </c>
       <c r="H62" s="24" t="inlineStr">
         <is>
-          <t>Fond, a little suggestive.</t>
+          <t>Angry.</t>
         </is>
       </c>
       <c r="I62" s="24" t="n"/>
@@ -13159,17 +13159,17 @@
       </c>
       <c r="B63" s="27" t="inlineStr">
         <is>
-          <t>hazel_fav_05</t>
+          <t>hazel_least_03</t>
         </is>
       </c>
       <c r="C63" s="26" t="inlineStr">
         <is>
-          <t>hazel_fav_05.wav</t>
+          <t>hazel_least_03.wav</t>
         </is>
       </c>
       <c r="D63" s="27" t="inlineStr">
         <is>
-          <t>Puzzle quip: you matched her favourite gem</t>
+          <t>Puzzle quip: you matched a gem she dislikes</t>
         </is>
       </c>
       <c r="E63" s="26" t="inlineStr">
@@ -13179,7 +13179,7 @@
       </c>
       <c r="F63" s="28" t="inlineStr">
         <is>
-          <t>Blossom. You have my attention.</t>
+          <t>No. I've seen what those do.</t>
         </is>
       </c>
       <c r="G63" s="27" t="inlineStr">
@@ -13189,7 +13189,7 @@
       </c>
       <c r="H63" s="27" t="inlineStr">
         <is>
-          <t>Dry, pleased.</t>
+          <t>Serious.</t>
         </is>
       </c>
       <c r="I63" s="27" t="n"/>
@@ -13201,17 +13201,17 @@
       </c>
       <c r="B64" s="24" t="inlineStr">
         <is>
-          <t>hazel_fav_06</t>
+          <t>hazel_least_04</t>
         </is>
       </c>
       <c r="C64" s="23" t="inlineStr">
         <is>
-          <t>hazel_fav_06.wav</t>
+          <t>hazel_least_04.wav</t>
         </is>
       </c>
       <c r="D64" s="24" t="inlineStr">
         <is>
-          <t>Puzzle quip: you matched her favourite gem</t>
+          <t>Puzzle quip: you matched a gem she dislikes</t>
         </is>
       </c>
       <c r="E64" s="23" t="inlineStr">
@@ -13221,17 +13221,17 @@
       </c>
       <c r="F64" s="25" t="inlineStr">
         <is>
-          <t>Don't stop on my account.</t>
+          <t>I'll pretend I didn't see that.</t>
         </is>
       </c>
       <c r="G64" s="24" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>angry</t>
         </is>
       </c>
       <c r="H64" s="24" t="inlineStr">
         <is>
-          <t>Warm.</t>
+          <t>Annoyed.</t>
         </is>
       </c>
       <c r="I64" s="24" t="n"/>
@@ -13243,15 +13243,15 @@
       </c>
       <c r="B65" s="27" t="inlineStr">
         <is>
-          <t>hazel_least_01</t>
+          <t>hazel_least_05</t>
         </is>
       </c>
       <c r="C65" s="26" t="inlineStr">
         <is>
-          <t>hazel_least_01.wav</t>
-        </is>
-      </c>
-      <c r="D65" s="28" t="inlineStr">
+          <t>hazel_least_05.wav</t>
+        </is>
+      </c>
+      <c r="D65" s="27" t="inlineStr">
         <is>
           <t>Puzzle quip: you matched a gem she dislikes</t>
         </is>
@@ -13263,7 +13263,7 @@
       </c>
       <c r="F65" s="28" t="inlineStr">
         <is>
-          <t>Fire. In a grove. Really?</t>
+          <t>Mind my leaves with that.</t>
         </is>
       </c>
       <c r="G65" s="27" t="inlineStr">
@@ -13273,7 +13273,7 @@
       </c>
       <c r="H65" s="27" t="inlineStr">
         <is>
-          <t>Calm disapproval.</t>
+          <t>Serious.</t>
         </is>
       </c>
       <c r="I65" s="27" t="n"/>
@@ -13285,17 +13285,17 @@
       </c>
       <c r="B66" s="24" t="inlineStr">
         <is>
-          <t>hazel_least_02</t>
+          <t>hazel_chat_01</t>
         </is>
       </c>
       <c r="C66" s="23" t="inlineStr">
         <is>
-          <t>hazel_least_02.wav</t>
-        </is>
-      </c>
-      <c r="D66" s="24" t="inlineStr">
-        <is>
-          <t>Puzzle quip: you matched a gem she dislikes</t>
+          <t>hazel_chat_01.wav</t>
+        </is>
+      </c>
+      <c r="D66" s="25" t="inlineStr">
+        <is>
+          <t>Puzzle quip: chatter while you play</t>
         </is>
       </c>
       <c r="E66" s="23" t="inlineStr">
@@ -13305,7 +13305,7 @@
       </c>
       <c r="F66" s="25" t="inlineStr">
         <is>
-          <t>Put that out.</t>
+          <t>Slower. I can hear you panicking.</t>
         </is>
       </c>
       <c r="G66" s="24" t="inlineStr">
@@ -13315,7 +13315,7 @@
       </c>
       <c r="H66" s="24" t="inlineStr">
         <is>
-          <t>Quiet order.</t>
+          <t>Teasing.</t>
         </is>
       </c>
       <c r="I66" s="24" t="n"/>
@@ -13327,17 +13327,17 @@
       </c>
       <c r="B67" s="27" t="inlineStr">
         <is>
-          <t>hazel_least_03</t>
+          <t>hazel_chat_02</t>
         </is>
       </c>
       <c r="C67" s="26" t="inlineStr">
         <is>
-          <t>hazel_least_03.wav</t>
+          <t>hazel_chat_02.wav</t>
         </is>
       </c>
       <c r="D67" s="27" t="inlineStr">
         <is>
-          <t>Puzzle quip: you matched a gem she dislikes</t>
+          <t>Puzzle quip: chatter while you play</t>
         </is>
       </c>
       <c r="E67" s="26" t="inlineStr">
@@ -13347,7 +13347,7 @@
       </c>
       <c r="F67" s="28" t="inlineStr">
         <is>
-          <t>No. I've seen what those do.</t>
+          <t>Forty years, I said. Mind where you swing.</t>
         </is>
       </c>
       <c r="G67" s="27" t="inlineStr">
@@ -13357,7 +13357,7 @@
       </c>
       <c r="H67" s="27" t="inlineStr">
         <is>
-          <t>Grim, short.</t>
+          <t>Teasing.</t>
         </is>
       </c>
       <c r="I67" s="27" t="n"/>
@@ -13369,17 +13369,17 @@
       </c>
       <c r="B68" s="24" t="inlineStr">
         <is>
-          <t>hazel_least_04</t>
+          <t>hazel_chat_04</t>
         </is>
       </c>
       <c r="C68" s="23" t="inlineStr">
         <is>
-          <t>hazel_least_04.wav</t>
+          <t>hazel_chat_04.wav</t>
         </is>
       </c>
       <c r="D68" s="24" t="inlineStr">
         <is>
-          <t>Puzzle quip: you matched a gem she dislikes</t>
+          <t>Puzzle quip: chatter while you play</t>
         </is>
       </c>
       <c r="E68" s="23" t="inlineStr">
@@ -13389,17 +13389,17 @@
       </c>
       <c r="F68" s="25" t="inlineStr">
         <is>
-          <t>Embers. I'll pretend I didn't see that.</t>
+          <t>You've got mud on your face. Leave it. It suits you.</t>
         </is>
       </c>
       <c r="G68" s="24" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>teasing</t>
         </is>
       </c>
       <c r="H68" s="24" t="inlineStr">
         <is>
-          <t>Dry.</t>
+          <t>Flirting.</t>
         </is>
       </c>
       <c r="I68" s="24" t="n"/>
@@ -13411,17 +13411,17 @@
       </c>
       <c r="B69" s="27" t="inlineStr">
         <is>
-          <t>hazel_least_05</t>
+          <t>hazel_chat_05</t>
         </is>
       </c>
       <c r="C69" s="26" t="inlineStr">
         <is>
-          <t>hazel_least_05.wav</t>
+          <t>hazel_chat_05.wav</t>
         </is>
       </c>
       <c r="D69" s="27" t="inlineStr">
         <is>
-          <t>Puzzle quip: you matched a gem she dislikes</t>
+          <t>Puzzle quip: chatter while you play</t>
         </is>
       </c>
       <c r="E69" s="26" t="inlineStr">
@@ -13431,7 +13431,7 @@
       </c>
       <c r="F69" s="28" t="inlineStr">
         <is>
-          <t>Mind my leaves with that.</t>
+          <t>Better than the last one the miller sent.</t>
         </is>
       </c>
       <c r="G69" s="27" t="inlineStr">
@@ -13441,7 +13441,7 @@
       </c>
       <c r="H69" s="27" t="inlineStr">
         <is>
-          <t>Calm warning.</t>
+          <t>Teasing.</t>
         </is>
       </c>
       <c r="I69" s="27" t="n"/>
@@ -13453,15 +13453,15 @@
       </c>
       <c r="B70" s="24" t="inlineStr">
         <is>
-          <t>hazel_chat_01</t>
+          <t>hazel_chat_06</t>
         </is>
       </c>
       <c r="C70" s="23" t="inlineStr">
         <is>
-          <t>hazel_chat_01.wav</t>
-        </is>
-      </c>
-      <c r="D70" s="25" t="inlineStr">
+          <t>hazel_chat_06.wav</t>
+        </is>
+      </c>
+      <c r="D70" s="24" t="inlineStr">
         <is>
           <t>Puzzle quip: chatter while you play</t>
         </is>
@@ -13473,7 +13473,7 @@
       </c>
       <c r="F70" s="25" t="inlineStr">
         <is>
-          <t>Slower. I can hear you panicking.</t>
+          <t>I'm not watching you. I'm photosynthesising.</t>
         </is>
       </c>
       <c r="G70" s="24" t="inlineStr">
@@ -13483,7 +13483,7 @@
       </c>
       <c r="H70" s="24" t="inlineStr">
         <is>
-          <t>Patient, dry.</t>
+          <t>Teasing.</t>
         </is>
       </c>
       <c r="I70" s="24" t="n"/>
@@ -13495,12 +13495,12 @@
       </c>
       <c r="B71" s="27" t="inlineStr">
         <is>
-          <t>hazel_chat_02</t>
+          <t>hazel_chat_07</t>
         </is>
       </c>
       <c r="C71" s="26" t="inlineStr">
         <is>
-          <t>hazel_chat_02.wav</t>
+          <t>hazel_chat_07.wav</t>
         </is>
       </c>
       <c r="D71" s="27" t="inlineStr">
@@ -13515,7 +13515,7 @@
       </c>
       <c r="F71" s="28" t="inlineStr">
         <is>
-          <t>Forty years, I said. Mind where you swing.</t>
+          <t>Take your time. I've got about three hundred years.</t>
         </is>
       </c>
       <c r="G71" s="27" t="inlineStr">
@@ -13525,313 +13525,19 @@
       </c>
       <c r="H71" s="27" t="inlineStr">
         <is>
-          <t>Dry reminder.</t>
+          <t>Calm.</t>
         </is>
       </c>
       <c r="I71" s="27" t="n"/>
       <c r="J71" s="27" t="n"/>
     </row>
-    <row r="72" ht="27" customHeight="1">
-      <c r="A72" s="23" t="n">
-        <v>67</v>
-      </c>
-      <c r="B72" s="24" t="inlineStr">
-        <is>
-          <t>hazel_chat_03</t>
-        </is>
-      </c>
-      <c r="C72" s="23" t="inlineStr">
-        <is>
-          <t>hazel_chat_03.wav</t>
-        </is>
-      </c>
-      <c r="D72" s="24" t="inlineStr">
-        <is>
-          <t>Puzzle quip: chatter while you play</t>
-        </is>
-      </c>
-      <c r="E72" s="23" t="inlineStr">
-        <is>
-          <t>Short bark, shown as a pop-up while you play.</t>
-        </is>
-      </c>
-      <c r="F72" s="25" t="inlineStr">
-        <is>
-          <t>The ferns are watching. Give them something to talk about.</t>
-        </is>
-      </c>
-      <c r="G72" s="24" t="inlineStr">
-        <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="H72" s="24" t="inlineStr">
-        <is>
-          <t>Sly.</t>
-        </is>
-      </c>
-      <c r="I72" s="24" t="n"/>
-      <c r="J72" s="24" t="n"/>
-    </row>
-    <row r="73" ht="27" customHeight="1">
-      <c r="A73" s="26" t="n">
-        <v>68</v>
-      </c>
-      <c r="B73" s="27" t="inlineStr">
-        <is>
-          <t>hazel_chat_04</t>
-        </is>
-      </c>
-      <c r="C73" s="26" t="inlineStr">
-        <is>
-          <t>hazel_chat_04.wav</t>
-        </is>
-      </c>
-      <c r="D73" s="27" t="inlineStr">
-        <is>
-          <t>Puzzle quip: chatter while you play</t>
-        </is>
-      </c>
-      <c r="E73" s="26" t="inlineStr">
-        <is>
-          <t>Short bark, shown as a pop-up while you play.</t>
-        </is>
-      </c>
-      <c r="F73" s="28" t="inlineStr">
-        <is>
-          <t>You've got mud on your face. Leave it. It suits you.</t>
-        </is>
-      </c>
-      <c r="G73" s="27" t="inlineStr">
-        <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="H73" s="27" t="inlineStr">
-        <is>
-          <t>Fond.</t>
-        </is>
-      </c>
-      <c r="I73" s="27" t="n"/>
-      <c r="J73" s="27" t="n"/>
-    </row>
-    <row r="74" ht="27" customHeight="1">
-      <c r="A74" s="23" t="n">
-        <v>69</v>
-      </c>
-      <c r="B74" s="24" t="inlineStr">
-        <is>
-          <t>hazel_chat_05</t>
-        </is>
-      </c>
-      <c r="C74" s="23" t="inlineStr">
-        <is>
-          <t>hazel_chat_05.wav</t>
-        </is>
-      </c>
-      <c r="D74" s="24" t="inlineStr">
-        <is>
-          <t>Puzzle quip: chatter while you play</t>
-        </is>
-      </c>
-      <c r="E74" s="23" t="inlineStr">
-        <is>
-          <t>Short bark, shown as a pop-up while you play.</t>
-        </is>
-      </c>
-      <c r="F74" s="25" t="inlineStr">
-        <is>
-          <t>Better than the last one Aldous sent. Prettier, too.</t>
-        </is>
-      </c>
-      <c r="G74" s="24" t="inlineStr">
-        <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="H74" s="24" t="inlineStr">
-        <is>
-          <t>Dry, fond.</t>
-        </is>
-      </c>
-      <c r="I74" s="24" t="n"/>
-      <c r="J74" s="24" t="n"/>
-    </row>
-    <row r="75" ht="27" customHeight="1">
-      <c r="A75" s="26" t="n">
-        <v>70</v>
-      </c>
-      <c r="B75" s="27" t="inlineStr">
-        <is>
-          <t>hazel_chat_06</t>
-        </is>
-      </c>
-      <c r="C75" s="26" t="inlineStr">
-        <is>
-          <t>hazel_chat_06.wav</t>
-        </is>
-      </c>
-      <c r="D75" s="27" t="inlineStr">
-        <is>
-          <t>Puzzle quip: chatter while you play</t>
-        </is>
-      </c>
-      <c r="E75" s="26" t="inlineStr">
-        <is>
-          <t>Short bark, shown as a pop-up while you play.</t>
-        </is>
-      </c>
-      <c r="F75" s="28" t="inlineStr">
-        <is>
-          <t>I'm not watching you. I'm photosynthesising.</t>
-        </is>
-      </c>
-      <c r="G75" s="27" t="inlineStr">
-        <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="H75" s="27" t="inlineStr">
-        <is>
-          <t>Deadpan lie.</t>
-        </is>
-      </c>
-      <c r="I75" s="27" t="n"/>
-      <c r="J75" s="27" t="n"/>
-    </row>
-    <row r="76" ht="27" customHeight="1">
-      <c r="A76" s="23" t="n">
-        <v>71</v>
-      </c>
-      <c r="B76" s="24" t="inlineStr">
-        <is>
-          <t>hazel_chat_07</t>
-        </is>
-      </c>
-      <c r="C76" s="23" t="inlineStr">
-        <is>
-          <t>hazel_chat_07.wav</t>
-        </is>
-      </c>
-      <c r="D76" s="24" t="inlineStr">
-        <is>
-          <t>Puzzle quip: chatter while you play</t>
-        </is>
-      </c>
-      <c r="E76" s="23" t="inlineStr">
-        <is>
-          <t>Short bark, shown as a pop-up while you play.</t>
-        </is>
-      </c>
-      <c r="F76" s="25" t="inlineStr">
-        <is>
-          <t>Take your time. I've got a few hundred years.</t>
-        </is>
-      </c>
-      <c r="G76" s="24" t="inlineStr">
-        <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="H76" s="24" t="inlineStr">
-        <is>
-          <t>Unhurried.</t>
-        </is>
-      </c>
-      <c r="I76" s="24" t="n"/>
-      <c r="J76" s="24" t="n"/>
-    </row>
-    <row r="77" ht="27" customHeight="1">
-      <c r="A77" s="26" t="n">
-        <v>72</v>
-      </c>
-      <c r="B77" s="27" t="inlineStr">
-        <is>
-          <t>hazel_chat_08</t>
-        </is>
-      </c>
-      <c r="C77" s="26" t="inlineStr">
-        <is>
-          <t>hazel_chat_08.wav</t>
-        </is>
-      </c>
-      <c r="D77" s="27" t="inlineStr">
-        <is>
-          <t>Puzzle quip: chatter while you play</t>
-        </is>
-      </c>
-      <c r="E77" s="26" t="inlineStr">
-        <is>
-          <t>Short bark, shown as a pop-up while you play.</t>
-        </is>
-      </c>
-      <c r="F77" s="28" t="inlineStr">
-        <is>
-          <t>If you see the miller, wave. It makes him nervous.</t>
-        </is>
-      </c>
-      <c r="G77" s="27" t="inlineStr">
-        <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="H77" s="27" t="inlineStr">
-        <is>
-          <t>Mischievous.</t>
-        </is>
-      </c>
-      <c r="I77" s="27" t="n"/>
-      <c r="J77" s="27" t="n"/>
-    </row>
-    <row r="78" ht="27" customHeight="1">
-      <c r="A78" s="23" t="n">
-        <v>73</v>
-      </c>
-      <c r="B78" s="24" t="inlineStr">
-        <is>
-          <t>hazel_chat_09</t>
-        </is>
-      </c>
-      <c r="C78" s="23" t="inlineStr">
-        <is>
-          <t>hazel_chat_09.wav</t>
-        </is>
-      </c>
-      <c r="D78" s="24" t="inlineStr">
-        <is>
-          <t>Puzzle quip: chatter while you play</t>
-        </is>
-      </c>
-      <c r="E78" s="23" t="inlineStr">
-        <is>
-          <t>Short bark, shown as a pop-up while you play.</t>
-        </is>
-      </c>
-      <c r="F78" s="25" t="inlineStr">
-        <is>
-          <t>The badgers think you're doing well. They're wrong, but it's sweet.</t>
-        </is>
-      </c>
-      <c r="G78" s="24" t="inlineStr">
-        <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="H78" s="24" t="inlineStr">
-        <is>
-          <t>Teasing.</t>
-        </is>
-      </c>
-      <c r="I78" s="24" t="n"/>
-      <c r="J78" s="24" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A5:J78"/>
+  <autoFilter ref="A5:J71"/>
   <mergeCells count="1">
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I6:I78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I6:I71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>